<commit_message>
Correct nine points in Case Study: A Paired Pre-Post Study
The paired t-test is cross-checked by Wilcoxon, which assumes roughly symmetric differences, and the sign test (p 2.5e-4). The unpaired test still detects the effect, more weakly (p 0.011). Most users (35 of 45) got faster, and two (U27, U45) got 17 to 19 s slower. dz of -0.92 is large on the scale of the differences, d is -0.55, and a quiz distractor that was also correct is replaced. The take-it-further notebook uses old-design time as the baseline and reads the order check as a practice effect, and the Notes give -9 s and Chapter 91.
</commit_message>
<xml_diff>
--- a/data/case-study-a-paired-pre-post-study--ux_redesign.xlsx
+++ b/data/case-study-a-paired-pre-post-study--ux_redesign.xlsx
@@ -1348,7 +1348,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Simulated within-subject UX study for a paired pre/post case study (Chapter 138).</t>
+          <t>Simulated within-subject UX study for a paired pre/post case study (Chapter 91), a realistic teaching dataset written for the book.</t>
         </is>
       </c>
     </row>
@@ -1369,14 +1369,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Most users improved a lot on the new design; a group of non-responders barely changed, so the paired differences are non-normal and Wilcoxon signed-rank is the robust test.</t>
+          <t>Most users improved a lot on the new design; a group of non-responders barely changed, so the paired differences are non-normal, and the paired t-test is best cross-checked with Wilcoxon signed-rank and the sign test.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>The new design is genuinely faster; the paired mean difference is about -12 seconds.</t>
+          <t>The new design is faster; the paired mean difference is about -9 seconds.</t>
         </is>
       </c>
     </row>

</xml_diff>